<commit_message>
Add v1.1 validation package, codebook v1.1.1, and Silver toxicant correction
</commit_message>
<xml_diff>
--- a/cardiac_organoid_arms.xlsx
+++ b/cardiac_organoid_arms.xlsx
@@ -2618,7 +2618,6 @@
           <t>10.1038/s41467-022-34730-7</t>
         </is>
       </c>
-      <c r="BB11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3002,7 +3001,6 @@
           <t>10.1038/s41467-022-34730-7</t>
         </is>
       </c>
-      <c r="BB13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4179,7 +4177,6 @@
           <t>10.1016/j.celrep.2023.112322</t>
         </is>
       </c>
-      <c r="BB20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -4323,7 +4320,6 @@
           <t>10.1016/j.celrep.2023.112322</t>
         </is>
       </c>
-      <c r="BB21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -4482,7 +4478,6 @@
           <t>10.1038/s44161-025-00669-3</t>
         </is>
       </c>
-      <c r="BB22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -4646,7 +4641,6 @@
           <t>10.1038/s44161-025-00669-3</t>
         </is>
       </c>
-      <c r="BB23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -7417,7 +7411,6 @@
           <t>10.1126/science.adu9375</t>
         </is>
       </c>
-      <c r="BB38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -7561,7 +7554,6 @@
           <t>10.1016/j.mtbio.2025.101566</t>
         </is>
       </c>
-      <c r="BB39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -7695,7 +7687,6 @@
           <t>10.1016/j.mtbio.2025.101566</t>
         </is>
       </c>
-      <c r="BB40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -8170,7 +8161,6 @@
           <t>10.1186/s13287-022-03215-1</t>
         </is>
       </c>
-      <c r="BB43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -8309,7 +8299,6 @@
           <t>10.1186/s13287-022-03215-1</t>
         </is>
       </c>
-      <c r="BB44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -8869,7 +8858,6 @@
           <t>10.1111/cpr.13631</t>
         </is>
       </c>
-      <c r="BB47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -9304,7 +9292,6 @@
           <t>10.1002/cpz1.461</t>
         </is>
       </c>
-      <c r="BB50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -9463,7 +9450,6 @@
           <t>10.1002/cpz1.767</t>
         </is>
       </c>
-      <c r="BB51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -9632,7 +9618,6 @@
           <t>10.1073/pnas.1707316114</t>
         </is>
       </c>
-      <c r="BB52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -9801,7 +9786,6 @@
           <t>10.1073/pnas.1707316114</t>
         </is>
       </c>
-      <c r="BB53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -9935,7 +9919,6 @@
           <t>10.1038/s41551-020-0539-4</t>
         </is>
       </c>
-      <c r="BB54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -10262,7 +10245,6 @@
           <t>10.1016/j.cell.2023.10.030</t>
         </is>
       </c>
-      <c r="BB56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -10426,7 +10408,6 @@
           <t>10.1016/j.cell.2023.10.030</t>
         </is>
       </c>
-      <c r="BB57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -10580,7 +10561,6 @@
           <t>10.1016/j.cell.2023.10.030</t>
         </is>
       </c>
-      <c r="BB58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -10749,7 +10729,6 @@
           <t>10.1016/j.cell.2023.10.030</t>
         </is>
       </c>
-      <c r="BB59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -11244,7 +11223,6 @@
           <t>10.1016/j.stem.2020.05.004</t>
         </is>
       </c>
-      <c r="BB62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -11403,7 +11381,6 @@
           <t>10.1016/j.stem.2020.05.004</t>
         </is>
       </c>
-      <c r="BB63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -11537,7 +11514,6 @@
           <t>10.3390/biomedicines9121952</t>
         </is>
       </c>
-      <c r="BB64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -11671,7 +11647,6 @@
           <t>10.3390/biomedicines9121952</t>
         </is>
       </c>
-      <c r="BB65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -11805,7 +11780,6 @@
           <t>10.3390/biomedicines9121952</t>
         </is>
       </c>
-      <c r="BB66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -11939,7 +11913,6 @@
           <t>10.3390/biomedicines9121952</t>
         </is>
       </c>
-      <c r="BB67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -12063,7 +12036,6 @@
           <t>10.1177/19373341251392244</t>
         </is>
       </c>
-      <c r="BB68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -12187,7 +12159,6 @@
           <t>10.1177/19373341251392244</t>
         </is>
       </c>
-      <c r="BB69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -12306,7 +12277,6 @@
           <t>10.1016/j.crmeth.2024.100798</t>
         </is>
       </c>
-      <c r="BB70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -12430,7 +12400,6 @@
           <t>10.1016/j.crmeth.2024.100798</t>
         </is>
       </c>
-      <c r="BB71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -12549,7 +12518,6 @@
           <t>10.1016/j.crmeth.2024.100798</t>
         </is>
       </c>
-      <c r="BB72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -12663,7 +12631,6 @@
           <t>10.1016/j.crmeth.2024.100798</t>
         </is>
       </c>
-      <c r="BB73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -12782,7 +12749,6 @@
           <t>10.1016/j.crmeth.2024.100798</t>
         </is>
       </c>
-      <c r="BB74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -12896,7 +12862,6 @@
           <t>10.1016/j.crmeth.2024.100798</t>
         </is>
       </c>
-      <c r="BB75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -13010,7 +12975,6 @@
           <t>10.1016/j.crmeth.2024.100798</t>
         </is>
       </c>
-      <c r="BB76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -13159,7 +13123,6 @@
           <t>10.1021/acsbiomaterials.2c01290</t>
         </is>
       </c>
-      <c r="BB77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -13308,7 +13271,6 @@
           <t>10.1021/acsbiomaterials.2c01290</t>
         </is>
       </c>
-      <c r="BB78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -13457,7 +13419,6 @@
           <t>10.1021/acsbiomaterials.2c01290</t>
         </is>
       </c>
-      <c r="BB79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -13606,7 +13567,6 @@
           <t>10.1021/acsbiomaterials.2c01290</t>
         </is>
       </c>
-      <c r="BB80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -13765,7 +13725,6 @@
           <t>10.7554/eLife.83532</t>
         </is>
       </c>
-      <c r="BB81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -13911,7 +13870,7 @@
       </c>
       <c r="AW82" t="inlineStr">
         <is>
-          <t>no value reported</t>
+          <t>toxicant dosed</t>
         </is>
       </c>
       <c r="AX82" t="inlineStr">
@@ -14087,7 +14046,6 @@
           <t>10.7554/eLife.83532</t>
         </is>
       </c>
-      <c r="BB83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -14241,7 +14199,6 @@
           <t>10.7554/eLife.83532</t>
         </is>
       </c>
-      <c r="BB84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -14395,7 +14352,6 @@
           <t>10.7554/eLife.83532</t>
         </is>
       </c>
-      <c r="BB85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">

</xml_diff>